<commit_message>
Use current progress IDs in workbook
</commit_message>
<xml_diff>
--- a/outputs/progress-map/gdm_nh1_progress_story_generation_map.xlsx
+++ b/outputs/progress-map/gdm_nh1_progress_story_generation_map.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="R4a34342b78634cdc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="R850a6a2911a34c44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progress_Map" sheetId="3" r:id="R909b268120434b38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GDM_Book1" sheetId="4" r:id="R0516d3794e5f41a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NH1" sheetId="5" r:id="Rc3555ce9345b4dfd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="6" r:id="R8b4fa95ad9c74005"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="Re1fcc1ee4add443c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="Rf37da0deaf824b96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progress_Map" sheetId="3" r:id="Rf5dbf19361e84255"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GDM_Book1" sheetId="4" r:id="Rf5551e34daf346af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NH1" sheetId="5" r:id="R86231265df114507"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="6" r:id="Reec4f784ee014a2c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -376,10 +376,10 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>レベル名ではなく、GDMとNH1それぞれの進捗ID範囲で本文生成を指定するためのExcelです。</x:v>
+        <x:v>レベル名ではなく、GDMとNH1それぞれの現在到達IDで本文生成を指定するためのExcelです。</x:v>
       </x:c>
       <x:c r="B2" s="6" t="str">
-        <x:v>レベル名ではなく、GDMとNH1それぞれの進捗ID範囲で本文生成を指定するためのExcelです。</x:v>
+        <x:v>レベル名ではなく、GDMとNH1それぞれの現在到達IDで本文生成を指定するためのExcelです。</x:v>
       </x:c>
     </x:row>
     <x:row r="3"/>
@@ -396,7 +396,7 @@
         <x:v>目的</x:v>
       </x:c>
       <x:c r="B5" s="21" t="str">
-        <x:v>GDMとNH1を「レベル」ではなく進捗IDで指定し、物語本文を生成するための台帳です。</x:v>
+        <x:v>GDMとNH1を「レベル」ではなく現在到達している進捗IDで指定し、物語本文を生成するための台帳です。</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -404,46 +404,54 @@
         <x:v>基本</x:v>
       </x:c>
       <x:c r="B6" s="21" t="str">
-        <x:v>物語生成指定シートで GDM Start/End ID と NH1 Start/End ID を指定します。</x:v>
+        <x:v>物語生成指定シートで GDM Current ID と NH1 Current ID を指定します。</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="21" t="str">
-        <x:v>GDM</x:v>
+        <x:v>Startの考え方</x:v>
       </x:c>
       <x:c r="B7" s="21" t="str">
-        <x:v>GDM-41-10 を一区切りとし、そのあたりから NH1 を併用開始する想定です。</x:v>
+        <x:v>GDMは常に最初のIDから開始します。NH1は未開始なら0を指定します。</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="21" t="str">
-        <x:v>NH1</x:v>
+        <x:v>GDM</x:v>
       </x:c>
       <x:c r="B8" s="21" t="str">
-        <x:v>NH1 Start/End ID を空欄にするとGDMのみで生成する想定です。</x:v>
+        <x:v>GDM-41-10 を一区切りとし、そのあたりから NH1 を併用開始する想定です。</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="21" t="str">
-        <x:v>名詞</x:v>
+        <x:v>NH1</x:v>
       </x:c>
       <x:c r="B9" s="21" t="str">
-        <x:v>ユーザー方針により、名詞は導入リスト外でも自然な物語に必要なら使用可です。</x:v>
+        <x:v>NH1 Current ID が0ならGDMのみ、NH1-...ならNH1の最初からそのIDまでを併用する想定です。</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="21" t="str">
-        <x:v>品質方針</x:v>
+        <x:v>名詞</x:v>
       </x:c>
       <x:c r="B10" s="21" t="str">
-        <x:v>4コマ漫画のように起承転結を持たせ、次の展開が気になり、最後は明るく終える本文を優先します。</x:v>
+        <x:v>ユーザー方針により、名詞は導入リスト外でも自然な物語に必要なら使用可です。</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="21" t="str">
+        <x:v>品質方針</x:v>
+      </x:c>
+      <x:c r="B11" s="21" t="str">
+        <x:v>4コマ漫画のように起承転結を持たせ、次の展開が気になり、最後は明るく終える本文を優先します。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="15" hidden="0" customHeight="1">
+      <x:c r="A12" s="21" t="str">
         <x:v>確認状態</x:v>
       </x:c>
-      <x:c r="B11" s="21" t="str">
+      <x:c r="B12" s="21" t="str">
         <x:v>docx内の文字は画像化されていたため、台帳の多くは画像から転記しています。原本更新時は確認状態列を見て補正してください。</x:v>
       </x:c>
     </x:row>
@@ -478,13 +486,13 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>B列を書き換えて、GDM/NH1の進捗ID範囲と物語条件を指定します。</x:v>
+        <x:v>B列を書き換えて、GDM/NH1の現在到達IDと物語条件を指定します。</x:v>
       </x:c>
       <x:c r="B2" s="6" t="str">
-        <x:v>B列を書き換えて、GDM/NH1の進捗ID範囲と物語条件を指定します。</x:v>
+        <x:v>B列を書き換えて、GDM/NH1の現在到達IDと物語条件を指定します。</x:v>
       </x:c>
       <x:c r="C2" s="6" t="str">
-        <x:v>B列を書き換えて、GDM/NH1の進捗ID範囲と物語条件を指定します。</x:v>
+        <x:v>B列を書き換えて、GDM/NH1の現在到達IDと物語条件を指定します。</x:v>
       </x:c>
     </x:row>
     <x:row r="3"/>
@@ -523,140 +531,122 @@
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="21" t="str">
-        <x:v>GDM Start ID</x:v>
+        <x:v>GDM Current ID</x:v>
       </x:c>
       <x:c r="B7" s="22" t="str">
-        <x:v>GDM-1</x:v>
+        <x:v>GDM-41-10</x:v>
       </x:c>
       <x:c r="C7" s="21" t="str">
-        <x:v>必須。GDMの開始進捗ID</x:v>
+        <x:v>必須。GDMは最初のIDからここまでを使用可</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="21" t="str">
-        <x:v>GDM End ID</x:v>
+        <x:v>NH1 Current ID</x:v>
       </x:c>
       <x:c r="B8" s="22" t="str">
-        <x:v>GDM-41-10</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C8" s="21" t="str">
-        <x:v>必須。ここまでのGDM導入項目を使用可</x:v>
+        <x:v>NH1未開始なら0。開始後は到達済みのNH1進捗IDを指定</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="21" t="str">
-        <x:v>NH1 Start ID</x:v>
-      </x:c>
-      <x:c r="B9" s="22" t="str"/>
+        <x:v>Target Words</x:v>
+      </x:c>
+      <x:c r="B9" s="22" t="n">
+        <x:v>250</x:v>
+      </x:c>
       <x:c r="C9" s="21" t="str">
-        <x:v>GDM-41-10以降で併用する場合に指定</x:v>
+        <x:v>本文のおおよその語数</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="21" t="str">
-        <x:v>NH1 End ID</x:v>
-      </x:c>
-      <x:c r="B10" s="22" t="str"/>
+        <x:v>Target Reader</x:v>
+      </x:c>
+      <x:c r="B10" s="22" t="str">
+        <x:v>中学生英語塾</x:v>
+      </x:c>
       <x:c r="C10" s="21" t="str">
-        <x:v>NH1を使う場合の終了ID</x:v>
+        <x:v>読者層</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="21" t="str">
-        <x:v>Target Words</x:v>
-      </x:c>
-      <x:c r="B11" s="22" t="n">
-        <x:v>250</x:v>
+        <x:v>Main Characters</x:v>
+      </x:c>
+      <x:c r="B11" s="22" t="str">
+        <x:v>Ken, Yui</x:v>
       </x:c>
       <x:c r="C11" s="21" t="str">
-        <x:v>本文のおおよその語数</x:v>
+        <x:v>日本人に性別が分かりやすい名前を優先</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="21" t="str">
-        <x:v>Target Reader</x:v>
+        <x:v>Age Range</x:v>
       </x:c>
       <x:c r="B12" s="22" t="str">
-        <x:v>中学生英語塾</x:v>
+        <x:v>12-15</x:v>
       </x:c>
       <x:c r="C12" s="21" t="str">
-        <x:v>読者層</x:v>
+        <x:v>話ごとに小学生から大人まで変えてよい</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="21" t="str">
-        <x:v>Main Characters</x:v>
+        <x:v>Setting</x:v>
       </x:c>
       <x:c r="B13" s="22" t="str">
-        <x:v>Ken, Yui</x:v>
+        <x:v>school / shop / station / festival</x:v>
       </x:c>
       <x:c r="C13" s="21" t="str">
-        <x:v>日本人に性別が分かりやすい名前を優先</x:v>
+        <x:v>舞台。話ごとに系統を変える</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="21" t="str">
-        <x:v>Age Range</x:v>
+        <x:v>Story Shape</x:v>
       </x:c>
       <x:c r="B14" s="22" t="str">
-        <x:v>12-15</x:v>
+        <x:v>4コマ的な起承転結</x:v>
       </x:c>
       <x:c r="C14" s="21" t="str">
-        <x:v>話ごとに小学生から大人まで変えてよい</x:v>
+        <x:v>暗すぎず、最後はハッピーにする</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="21" t="str">
-        <x:v>Setting</x:v>
+        <x:v>Noun Policy</x:v>
       </x:c>
       <x:c r="B15" s="22" t="str">
-        <x:v>school / shop / station / festival</x:v>
+        <x:v>名詞はリスト外でも必要なら可</x:v>
       </x:c>
       <x:c r="C15" s="21" t="str">
-        <x:v>舞台。話ごとに系統を変える</x:v>
+        <x:v>ただし動詞・文法は進捗IDに沿う</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="21" t="str">
-        <x:v>Story Shape</x:v>
+        <x:v>Tone</x:v>
       </x:c>
       <x:c r="B16" s="22" t="str">
-        <x:v>4コマ的な起承転結</x:v>
+        <x:v>次の展開が気になる / 明るい結末</x:v>
       </x:c>
       <x:c r="C16" s="21" t="str">
-        <x:v>暗すぎず、最後はハッピーにする</x:v>
+        <x:v>ミステリー可。救いのある終わりにする</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="21" t="str">
-        <x:v>Noun Policy</x:v>
+        <x:v>Output</x:v>
       </x:c>
       <x:c r="B17" s="22" t="str">
-        <x:v>名詞はリスト外でも必要なら可</x:v>
+        <x:v>plain text first</x:v>
       </x:c>
       <x:c r="C17" s="21" t="str">
-        <x:v>ただし動詞・文法は進捗IDに沿う</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="15" hidden="0" customHeight="1">
-      <x:c r="A18" s="21" t="str">
-        <x:v>Tone</x:v>
-      </x:c>
-      <x:c r="B18" s="22" t="str">
-        <x:v>次の展開が気になる / 明るい結末</x:v>
-      </x:c>
-      <x:c r="C18" s="21" t="str">
-        <x:v>ミステリー可。救いのある終わりにする</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="15" hidden="0" customHeight="1">
-      <x:c r="A19" s="21" t="str">
-        <x:v>Output</x:v>
-      </x:c>
-      <x:c r="B19" s="22" t="str">
-        <x:v>plain text first</x:v>
-      </x:c>
-      <x:c r="C19" s="21" t="str">
         <x:v>画像は後工程。本文品質を優先</x:v>
       </x:c>
     </x:row>
@@ -719,34 +709,34 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>GDMとNH1を同じ形式で並べたマスター表です。指定範囲に含まれるIDの導入項目を本文生成に使います。</x:v>
+        <x:v>GDMとNH1を同じ形式で並べたマスター表です。現在到達IDまでの導入項目を本文生成に使います。</x:v>
       </x:c>
       <x:c r="B2" s="6" t="str">
-        <x:v>GDMとNH1を同じ形式で並べたマスター表です。指定範囲に含まれるIDの導入項目を本文生成に使います。</x:v>
+        <x:v>GDMとNH1を同じ形式で並べたマスター表です。現在到達IDまでの導入項目を本文生成に使います。</x:v>
       </x:c>
       <x:c r="C2" s="6" t="str">
-        <x:v>GDMとNH1を同じ形式で並べたマスター表です。指定範囲に含まれるIDの導入項目を本文生成に使います。</x:v>
+        <x:v>GDMとNH1を同じ形式で並べたマスター表です。現在到達IDまでの導入項目を本文生成に使います。</x:v>
       </x:c>
       <x:c r="D2" s="6" t="str">
-        <x:v>GDMとNH1を同じ形式で並べたマスター表です。指定範囲に含まれるIDの導入項目を本文生成に使います。</x:v>
+        <x:v>GDMとNH1を同じ形式で並べたマスター表です。現在到達IDまでの導入項目を本文生成に使います。</x:v>
       </x:c>
       <x:c r="E2" s="6" t="str">
-        <x:v>GDMとNH1を同じ形式で並べたマスター表です。指定範囲に含まれるIDの導入項目を本文生成に使います。</x:v>
+        <x:v>GDMとNH1を同じ形式で並べたマスター表です。現在到達IDまでの導入項目を本文生成に使います。</x:v>
       </x:c>
       <x:c r="F2" s="6" t="str">
-        <x:v>GDMとNH1を同じ形式で並べたマスター表です。指定範囲に含まれるIDの導入項目を本文生成に使います。</x:v>
+        <x:v>GDMとNH1を同じ形式で並べたマスター表です。現在到達IDまでの導入項目を本文生成に使います。</x:v>
       </x:c>
       <x:c r="G2" s="6" t="str">
-        <x:v>GDMとNH1を同じ形式で並べたマスター表です。指定範囲に含まれるIDの導入項目を本文生成に使います。</x:v>
+        <x:v>GDMとNH1を同じ形式で並べたマスター表です。現在到達IDまでの導入項目を本文生成に使います。</x:v>
       </x:c>
       <x:c r="H2" s="6" t="str">
-        <x:v>GDMとNH1を同じ形式で並べたマスター表です。指定範囲に含まれるIDの導入項目を本文生成に使います。</x:v>
+        <x:v>GDMとNH1を同じ形式で並べたマスター表です。現在到達IDまでの導入項目を本文生成に使います。</x:v>
       </x:c>
       <x:c r="I2" s="6" t="str">
-        <x:v>GDMとNH1を同じ形式で並べたマスター表です。指定範囲に含まれるIDの導入項目を本文生成に使います。</x:v>
+        <x:v>GDMとNH1を同じ形式で並べたマスター表です。現在到達IDまでの導入項目を本文生成に使います。</x:v>
       </x:c>
       <x:c r="J2" s="6" t="str">
-        <x:v>GDMとNH1を同じ形式で並べたマスター表です。指定範囲に含まれるIDの導入項目を本文生成に使います。</x:v>
+        <x:v>GDMとNH1を同じ形式で並べたマスター表です。現在到達IDまでの導入項目を本文生成に使います。</x:v>
       </x:c>
     </x:row>
     <x:row r="3"/>
@@ -14757,7 +14747,7 @@
         <x:v>生成指示</x:v>
       </x:c>
       <x:c r="B5" s="21" t="str">
-        <x:v>GDM進捗ID {GDM Start ID} から {GDM End ID} まで、必要ならNH1進捗ID {NH1 Start ID} から {NH1 End ID} までを使用して、中学生向け英語リーディング本文を作る。</x:v>
+        <x:v>GDMは最初のIDから {GDM Current ID} までを使用する。NH1 Current ID が0ならNH1は使わず、NH1-...ならNH1の最初から {NH1 Current ID} までを併用して、中学生向け英語リーディング本文を作る。</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -14765,7 +14755,7 @@
         <x:v>語彙制約</x:v>
       </x:c>
       <x:c r="B6" s="21" t="str">
-        <x:v>動詞・文法・機能語は指定範囲を優先する。名詞は自然な物語に必要なら未導入でも使用可。</x:v>
+        <x:v>動詞・文法・機能語は指定された到達IDまでを優先する。名詞は自然な物語に必要なら未導入でも使用可。</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -14789,7 +14779,7 @@
         <x:v>出力</x:v>
       </x:c>
       <x:c r="B9" s="21" t="str">
-        <x:v>タイトル、想定進捗ID範囲、本文、語数、使用した主な導入項目メモを出す。</x:v>
+        <x:v>タイトル、GDM Current ID、NH1 Current ID、本文、語数、使用した主な導入項目メモを出す。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Map readings to current progress IDs
</commit_message>
<xml_diff>
--- a/outputs/progress-map/gdm_nh1_progress_story_generation_map.xlsx
+++ b/outputs/progress-map/gdm_nh1_progress_story_generation_map.xlsx
@@ -2,12 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="Re1fcc1ee4add443c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="Rf37da0deaf824b96"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progress_Map" sheetId="3" r:id="Rf5dbf19361e84255"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GDM_Book1" sheetId="4" r:id="Rf5551e34daf346af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NH1" sheetId="5" r:id="R86231265df114507"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="6" r:id="Reec4f784ee014a2c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="R5260ec73fe734ab1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="Rbfc754060e704447"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progress_Map" sheetId="3" r:id="Re5ee6ae15c274a6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GDM_Book1" sheetId="4" r:id="Rd31df0691fcb41c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NH1" sheetId="5" r:id="R1f788b631ca34f87"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="6" r:id="Rc1c97780224540d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Existing_Content_Map" sheetId="7" r:id="R782e058a2108488c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -433,25 +434,33 @@
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="21" t="str">
-        <x:v>名詞</x:v>
+        <x:v>既存コンテンツ</x:v>
       </x:c>
       <x:c r="B10" s="21" t="str">
-        <x:v>ユーザー方針により、名詞は導入リスト外でも自然な物語に必要なら使用可です。</x:v>
+        <x:v>Existing_Content_Map シートで、現在サイトにあるLevel 1-6本文のAssumed gradingとCurrent ID対応を確認できます。</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="21" t="str">
-        <x:v>品質方針</x:v>
+        <x:v>名詞</x:v>
       </x:c>
       <x:c r="B11" s="21" t="str">
-        <x:v>4コマ漫画のように起承転結を持たせ、次の展開が気になり、最後は明るく終える本文を優先します。</x:v>
+        <x:v>ユーザー方針により、名詞は導入リスト外でも自然な物語に必要なら使用可です。</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="21" t="str">
+        <x:v>品質方針</x:v>
+      </x:c>
+      <x:c r="B12" s="21" t="str">
+        <x:v>4コマ漫画のように起承転結を持たせ、次の展開が気になり、最後は明るく終える本文を優先します。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
+      <x:c r="A13" s="21" t="str">
         <x:v>確認状態</x:v>
       </x:c>
-      <x:c r="B12" s="21" t="str">
+      <x:c r="B13" s="21" t="str">
         <x:v>docx内の文字は画像化されていたため、台帳の多くは画像から転記しています。原本更新時は確認状態列を見て補正してください。</x:v>
       </x:c>
     </x:row>
@@ -14789,4 +14798,184 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="82" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="52" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="19.200000762939453" hidden="0" customHeight="1">
+      <x:c r="A1" s="4" t="str">
+        <x:v>既存コンテンツ Current ID 対応</x:v>
+      </x:c>
+      <x:c r="B1" s="4" t="str">
+        <x:v>既存コンテンツ Current ID 対応</x:v>
+      </x:c>
+      <x:c r="C1" s="4" t="str">
+        <x:v>既存コンテンツ Current ID 対応</x:v>
+      </x:c>
+      <x:c r="D1" s="4" t="str">
+        <x:v>既存コンテンツ Current ID 対応</x:v>
+      </x:c>
+      <x:c r="E1" s="4" t="str">
+        <x:v>既存コンテンツ Current ID 対応</x:v>
+      </x:c>
+      <x:c r="F1" s="4" t="str">
+        <x:v>既存コンテンツ Current ID 対応</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2" s="6" t="str">
+        <x:v>現在サイトに入っているLevel 1-6本文のAssumed gradingを、GDM/NH1 Current IDに対応づけた表です。</x:v>
+      </x:c>
+      <x:c r="B2" s="6" t="str">
+        <x:v>現在サイトに入っているLevel 1-6本文のAssumed gradingを、GDM/NH1 Current IDに対応づけた表です。</x:v>
+      </x:c>
+      <x:c r="C2" s="6" t="str">
+        <x:v>現在サイトに入っているLevel 1-6本文のAssumed gradingを、GDM/NH1 Current IDに対応づけた表です。</x:v>
+      </x:c>
+      <x:c r="D2" s="6" t="str">
+        <x:v>現在サイトに入っているLevel 1-6本文のAssumed gradingを、GDM/NH1 Current IDに対応づけた表です。</x:v>
+      </x:c>
+      <x:c r="E2" s="6" t="str">
+        <x:v>現在サイトに入っているLevel 1-6本文のAssumed gradingを、GDM/NH1 Current IDに対応づけた表です。</x:v>
+      </x:c>
+      <x:c r="F2" s="6" t="str">
+        <x:v>現在サイトに入っているLevel 1-6本文のAssumed gradingを、GDM/NH1 Current IDに対応づけた表です。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3"/>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="20" t="str">
+        <x:v>Level</x:v>
+      </x:c>
+      <x:c r="B4" s="20" t="str">
+        <x:v>GDM Current ID</x:v>
+      </x:c>
+      <x:c r="C4" s="20" t="str">
+        <x:v>NH1 Current ID</x:v>
+      </x:c>
+      <x:c r="D4" s="20" t="str">
+        <x:v>Assumed grading</x:v>
+      </x:c>
+      <x:c r="E4" s="20" t="str">
+        <x:v>対応メモ</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
+      <x:c r="A5" s="21" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B5" s="21" t="str">
+        <x:v>GDM-41-10</x:v>
+      </x:c>
+      <x:c r="C5" s="21" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D5" s="21" t="str">
+        <x:v>very short present sentences, be/have/see/open/go, this/it, basic prepositions, simple nouns.</x:v>
+      </x:c>
+      <x:c r="E5" s="21" t="str">
+        <x:v>see まとめまで。NH1は未開始。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="21" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B6" s="21" t="str">
+        <x:v>GDM-42-4</x:v>
+      </x:c>
+      <x:c r="C6" s="21" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D6" s="21" t="str">
+        <x:v>Level 1 plus longer present sequences, basic questions, says/asks, not/no, repeated nouns.</x:v>
+      </x:c>
+      <x:c r="E6" s="21" t="str">
+        <x:v>say まで。現在形の会話と基本疑問を想定。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
+      <x:c r="A7" s="21" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B7" s="21" t="str">
+        <x:v>GDM-60-1</x:v>
+      </x:c>
+      <x:c r="C7" s="21" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D7" s="21" t="str">
+        <x:v>Level 2 plus basic past forms, said/saw/came/opened/took, did not, simple dialogue.</x:v>
+      </x:c>
+      <x:c r="E7" s="21" t="str">
+        <x:v>come まで。過去形・did not・移動を含む現行本文に合わせる。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="21" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B8" s="21" t="str">
+        <x:v>GDM-82</x:v>
+      </x:c>
+      <x:c r="C8" s="21" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D8" s="21" t="str">
+        <x:v>Level 3 plus there was/were, before/after, careful observation, simple reveal.</x:v>
+      </x:c>
+      <x:c r="E8" s="21" t="str">
+        <x:v>before/after と when question までを想定。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="21" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B9" s="21" t="str">
+        <x:v>GDM-83</x:v>
+      </x:c>
+      <x:c r="C9" s="21" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D9" s="21" t="str">
+        <x:v>Level 4 plus fuller scenes, reason links, more characters, clearer resolution.</x:v>
+      </x:c>
+      <x:c r="E9" s="21" t="str">
+        <x:v>nothing/something まで。伏線と解決を少し増やす。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="21" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B10" s="21" t="str">
+        <x:v>GDM-106</x:v>
+      </x:c>
+      <x:c r="C10" s="21" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D10" s="21" t="str">
+        <x:v>Level 5 plus longer paragraphs, callbacks, multi-scene resolution, richer ending.</x:v>
+      </x:c>
+      <x:c r="E10" s="21" t="str">
+        <x:v>different/the same 付近まで。現行の長め本文を読む想定。</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:F1"/>
+    <x:mergeCell ref="A2:F2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add final ID genre readings
</commit_message>
<xml_diff>
--- a/outputs/progress-map/gdm_nh1_progress_story_generation_map.xlsx
+++ b/outputs/progress-map/gdm_nh1_progress_story_generation_map.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="R5260ec73fe734ab1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="Rbfc754060e704447"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progress_Map" sheetId="3" r:id="Re5ee6ae15c274a6d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GDM_Book1" sheetId="4" r:id="Rd31df0691fcb41c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NH1" sheetId="5" r:id="R1f788b631ca34f87"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="6" r:id="Rc1c97780224540d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Existing_Content_Map" sheetId="7" r:id="R782e058a2108488c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="R098cd0f921b04d04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="Ra650a16beb81449e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progress_Map" sheetId="3" r:id="R8f6f62a615044df9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GDM_Book1" sheetId="4" r:id="R29eab8ac8a7b4540"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NH1" sheetId="5" r:id="R0ff5e6747ba247f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="6" r:id="R87d3cfb9c52f426e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Existing_Content_Map" sheetId="7" r:id="R3c8eeb04544547d8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -437,7 +437,7 @@
         <x:v>既存コンテンツ</x:v>
       </x:c>
       <x:c r="B10" s="21" t="str">
-        <x:v>Existing_Content_Map シートで、現在サイトにあるLevel 1-6本文のAssumed gradingとCurrent ID対応を確認できます。</x:v>
+        <x:v>Existing_Content_Map シートで、現在サイトにあるLevel 1-7本文のAssumed gradingとCurrent ID対応を確認できます。</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
@@ -14833,22 +14833,22 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>現在サイトに入っているLevel 1-6本文のAssumed gradingを、GDM/NH1 Current IDに対応づけた表です。</x:v>
+        <x:v>現在サイトに入っているLevel 1-7本文のAssumed gradingを、GDM/NH1 Current IDに対応づけた表です。</x:v>
       </x:c>
       <x:c r="B2" s="6" t="str">
-        <x:v>現在サイトに入っているLevel 1-6本文のAssumed gradingを、GDM/NH1 Current IDに対応づけた表です。</x:v>
+        <x:v>現在サイトに入っているLevel 1-7本文のAssumed gradingを、GDM/NH1 Current IDに対応づけた表です。</x:v>
       </x:c>
       <x:c r="C2" s="6" t="str">
-        <x:v>現在サイトに入っているLevel 1-6本文のAssumed gradingを、GDM/NH1 Current IDに対応づけた表です。</x:v>
+        <x:v>現在サイトに入っているLevel 1-7本文のAssumed gradingを、GDM/NH1 Current IDに対応づけた表です。</x:v>
       </x:c>
       <x:c r="D2" s="6" t="str">
-        <x:v>現在サイトに入っているLevel 1-6本文のAssumed gradingを、GDM/NH1 Current IDに対応づけた表です。</x:v>
+        <x:v>現在サイトに入っているLevel 1-7本文のAssumed gradingを、GDM/NH1 Current IDに対応づけた表です。</x:v>
       </x:c>
       <x:c r="E2" s="6" t="str">
-        <x:v>現在サイトに入っているLevel 1-6本文のAssumed gradingを、GDM/NH1 Current IDに対応づけた表です。</x:v>
+        <x:v>現在サイトに入っているLevel 1-7本文のAssumed gradingを、GDM/NH1 Current IDに対応づけた表です。</x:v>
       </x:c>
       <x:c r="F2" s="6" t="str">
-        <x:v>現在サイトに入っているLevel 1-6本文のAssumed gradingを、GDM/NH1 Current IDに対応づけた表です。</x:v>
+        <x:v>現在サイトに入っているLevel 1-7本文のAssumed gradingを、GDM/NH1 Current IDに対応づけた表です。</x:v>
       </x:c>
     </x:row>
     <x:row r="3"/>
@@ -14969,6 +14969,23 @@
       </x:c>
       <x:c r="E10" s="21" t="str">
         <x:v>different/the same 付近まで。現行の長め本文を読む想定。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="24" hidden="0" customHeight="1">
+      <x:c r="A11" s="21" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B11" s="21" t="str">
+        <x:v>GDM-198</x:v>
+      </x:c>
+      <x:c r="C11" s="21" t="str">
+        <x:v>NH1-1-11-1-MAYBE</x:v>
+      </x:c>
+      <x:c r="D11" s="21" t="str">
+        <x:v>final GDM and NH1 IDs, longer scenes, stronger genre voice, clear comic or emotional resolution.</x:v>
+      </x:c>
+      <x:c r="E11" s="21" t="str">
+        <x:v>SF/Fantasy/Comedy の最終ID到達後本文。GDMとNH1の最終IDを併用する想定。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Add targeted level 3 comedy reading
</commit_message>
<xml_diff>
--- a/outputs/progress-map/gdm_nh1_progress_story_generation_map.xlsx
+++ b/outputs/progress-map/gdm_nh1_progress_story_generation_map.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="R098cd0f921b04d04"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="Ra650a16beb81449e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progress_Map" sheetId="3" r:id="R8f6f62a615044df9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GDM_Book1" sheetId="4" r:id="R29eab8ac8a7b4540"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NH1" sheetId="5" r:id="R0ff5e6747ba247f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="6" r:id="R87d3cfb9c52f426e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Existing_Content_Map" sheetId="7" r:id="R3c8eeb04544547d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="R6a02f7b5f5e8430b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="R1db5a11144d44f1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progress_Map" sheetId="3" r:id="R3f2f3d41b6f848b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GDM_Book1" sheetId="4" r:id="Rfb7829327c9e4150"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NH1" sheetId="5" r:id="R0ee4d1b527934552"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="6" r:id="Re539014edf7f4529"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Existing_Content_Map" sheetId="7" r:id="R118711df6c0b42f2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14903,7 +14903,7 @@
         <x:v>say まで。現在形の会話と基本疑問を想定。</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="15" hidden="0" customHeight="1">
+    <x:row r="7" ht="24" hidden="0" customHeight="1">
       <x:c r="A7" s="21" t="n">
         <x:v>3</x:v>
       </x:c>
@@ -14911,13 +14911,13 @@
         <x:v>GDM-60-1</x:v>
       </x:c>
       <x:c r="C7" s="21" t="str">
-        <x:v>0</x:v>
+        <x:v>NH1-1-5-2</x:v>
       </x:c>
       <x:c r="D7" s="21" t="str">
-        <x:v>Level 2 plus basic past forms, said/saw/came/opened/took, did not, simple dialogue.</x:v>
+        <x:v>Level 2 plus basic past forms, said/saw/came/opened/took, did not, simple dialogue. Required target items include come, Don't be, Let's, something/nothing, and How.</x:v>
       </x:c>
       <x:c r="E7" s="21" t="str">
-        <x:v>come まで。過去形・did not・移動を含む現行本文に合わせる。</x:v>
+        <x:v>GDM-60-1 の come と、NH1-1-5-2 の Don't be / Let's / something / nothing / How を必ず入れる。</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">

</xml_diff>